<commit_message>
Add função de conceder permissão de leitura nas pastas do drive quando convida uma pessoa (individual e em massa).
</commit_message>
<xml_diff>
--- a/modelos/modelo_convite_pessoas_em_massa.xlsx
+++ b/modelos/modelo_convite_pessoas_em_massa.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t xml:space="preserve">nome_completo</t>
   </si>
@@ -35,30 +35,6 @@
   </si>
   <si>
     <t xml:space="preserve">projetos (códigos separados por vírgula) (opcional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toni Garrido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">técnico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">renato@ispn.org.br</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cod/04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toni Beloto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jenipapos@yahoo.com.br</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paulo Miklos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">renato@renato.org.br</t>
   </si>
 </sst>
 </file>
@@ -172,7 +148,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.76"/>
@@ -199,50 +175,12 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="0" t="n">
-        <v>666666</v>
-      </c>
-      <c r="E2" s="0" t="s">
-        <v>8</v>
-      </c>
+      <c r="A2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="0" t="n">
-        <v>55555</v>
-      </c>
+      <c r="A3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="0" t="n">
-        <v>44444</v>
-      </c>
-    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>